<commit_message>
Create models.py and init_default_data.py Delete current_proforma_schedule display Change proforma_schedule -> current_proforma
</commit_message>
<xml_diff>
--- a/data/rdr.xlsx
+++ b/data/rdr.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\django\PFSPoc\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A8ABBDF-803D-4403-8621-D0FC3F25818C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE635F3D-C4F2-4EAC-A1D4-2E3B311412F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9A544EAD-84AA-4D4C-8554-96B67EC8D31F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9A544EAD-84AA-4D4C-8554-96B67EC8D31F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="64">
   <si>
     <t>POD</t>
   </si>
@@ -874,10 +874,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DE3F23E-86BD-4EE4-8A59-D3B5A53FC95C}">
-  <dimension ref="C1:AL31"/>
+  <dimension ref="C1:AJ31"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999"/>
   <sheetData>
-    <row r="1" spans="3:38" ht="18" thickBot="1">
+    <row r="1" spans="3:36" ht="18" thickBot="1">
       <c r="C1" t="s">
         <v>63</v>
       </c>
@@ -897,39 +897,37 @@
       <c r="K1" s="7"/>
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="9" t="s">
+      <c r="N1" s="8"/>
+      <c r="O1" s="9" t="s">
         <v>4</v>
       </c>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
       <c r="R1" s="10"/>
       <c r="S1" s="10"/>
       <c r="T1" s="10"/>
       <c r="U1" s="10"/>
       <c r="V1" s="10"/>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
-      <c r="Y1" s="11"/>
-      <c r="Z1" s="12" t="s">
+      <c r="W1" s="11"/>
+      <c r="X1" s="12" t="s">
         <v>5</v>
       </c>
+      <c r="Y1" s="13"/>
+      <c r="Z1" s="13"/>
       <c r="AA1" s="13"/>
       <c r="AB1" s="13"/>
       <c r="AC1" s="13"/>
       <c r="AD1" s="13"/>
-      <c r="AE1" s="13"/>
-      <c r="AF1" s="13"/>
-      <c r="AG1" s="14"/>
-      <c r="AH1" s="15" t="s">
+      <c r="AE1" s="14"/>
+      <c r="AF1" s="15" t="s">
         <v>6</v>
       </c>
+      <c r="AG1" s="16"/>
+      <c r="AH1" s="16"/>
       <c r="AI1" s="16"/>
-      <c r="AJ1" s="16"/>
-      <c r="AK1" s="16"/>
-      <c r="AL1" s="17"/>
+      <c r="AJ1" s="17"/>
     </row>
-    <row r="2" spans="3:38" ht="18" thickBot="1">
+    <row r="2" spans="3:36" ht="18" thickBot="1">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -964,87 +962,81 @@
         <v>17</v>
       </c>
       <c r="N2" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="O2" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="P2" s="21" t="s">
         <v>18</v>
       </c>
+      <c r="O2" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="P2" s="22" t="s">
+        <v>20</v>
+      </c>
       <c r="Q2" s="22" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="R2" s="22" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="S2" s="22" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="T2" s="22" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="U2" s="22" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="V2" s="22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="W2" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="X2" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="Y2" s="22" t="s">
         <v>27</v>
       </c>
+      <c r="X2" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y2" s="23" t="s">
+        <v>29</v>
+      </c>
       <c r="Z2" s="23" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="AA2" s="23" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="AB2" s="23" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="AC2" s="23" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="AD2" s="23" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="AE2" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF2" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG2" s="23" t="s">
         <v>35</v>
       </c>
+      <c r="AF2" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG2" s="24" t="s">
+        <v>37</v>
+      </c>
       <c r="AH2" s="24" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="AI2" s="24" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="AJ2" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="AK2" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL2" s="24" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="3:38" ht="18" thickBot="1">
+    <row r="3" spans="3:36" ht="18" thickBot="1">
       <c r="C3" s="18" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="3:38" ht="18" thickBot="1">
+    <row r="4" spans="3:36" ht="18" thickBot="1">
       <c r="C4" s="25" t="s">
         <v>41</v>
       </c>
@@ -1079,19 +1071,19 @@
         <v>182</v>
       </c>
       <c r="N4" s="21">
-        <v>130</v>
-      </c>
-      <c r="O4" s="21">
-        <v>130</v>
-      </c>
-      <c r="P4" s="21">
-        <v>78</v>
+        <v>78</v>
+      </c>
+      <c r="O4" s="22">
+        <v>828</v>
+      </c>
+      <c r="P4" s="22">
+        <v>342</v>
       </c>
       <c r="Q4" s="22">
-        <v>828</v>
+        <v>0</v>
       </c>
       <c r="R4" s="22">
-        <v>342</v>
+        <v>0</v>
       </c>
       <c r="S4" s="22">
         <v>0</v>
@@ -1100,19 +1092,19 @@
         <v>0</v>
       </c>
       <c r="U4" s="22">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="V4" s="22">
         <v>0</v>
       </c>
       <c r="W4" s="22">
-        <v>71</v>
-      </c>
-      <c r="X4" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="22">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="X4" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y4" s="23">
+        <v>78</v>
       </c>
       <c r="Z4" s="23">
         <v>156</v>
@@ -1124,19 +1116,19 @@
         <v>156</v>
       </c>
       <c r="AC4" s="23">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="AD4" s="23">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="AE4" s="23">
-        <v>109</v>
-      </c>
-      <c r="AF4" s="23">
-        <v>78</v>
-      </c>
-      <c r="AG4" s="23">
-        <v>78</v>
+        <v>78</v>
+      </c>
+      <c r="AF4" s="24">
+        <v>125</v>
+      </c>
+      <c r="AG4" s="24">
+        <v>62</v>
       </c>
       <c r="AH4" s="24">
         <v>125</v>
@@ -1147,14 +1139,8 @@
       <c r="AJ4" s="24">
         <v>125</v>
       </c>
-      <c r="AK4" s="24">
-        <v>62</v>
-      </c>
-      <c r="AL4" s="24">
-        <v>125</v>
-      </c>
     </row>
-    <row r="5" spans="3:38" ht="18" thickBot="1">
+    <row r="5" spans="3:36" ht="18" thickBot="1">
       <c r="C5" s="25" t="s">
         <v>42</v>
       </c>
@@ -1189,19 +1175,19 @@
         <v>182</v>
       </c>
       <c r="N5" s="21">
-        <v>130</v>
-      </c>
-      <c r="O5" s="21">
-        <v>130</v>
-      </c>
-      <c r="P5" s="21">
-        <v>78</v>
+        <v>78</v>
+      </c>
+      <c r="O5" s="22">
+        <v>44</v>
+      </c>
+      <c r="P5" s="22">
+        <v>28</v>
       </c>
       <c r="Q5" s="22">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="R5" s="22">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="S5" s="22">
         <v>0</v>
@@ -1210,19 +1196,19 @@
         <v>0</v>
       </c>
       <c r="U5" s="22">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="V5" s="22">
         <v>0</v>
       </c>
       <c r="W5" s="22">
-        <v>15</v>
-      </c>
-      <c r="X5" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="22">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="X5" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y5" s="23">
+        <v>78</v>
       </c>
       <c r="Z5" s="23">
         <v>156</v>
@@ -1234,19 +1220,19 @@
         <v>156</v>
       </c>
       <c r="AC5" s="23">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="AD5" s="23">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="AE5" s="23">
-        <v>109</v>
-      </c>
-      <c r="AF5" s="23">
-        <v>78</v>
-      </c>
-      <c r="AG5" s="23">
-        <v>78</v>
+        <v>78</v>
+      </c>
+      <c r="AF5" s="24">
+        <v>125</v>
+      </c>
+      <c r="AG5" s="24">
+        <v>62</v>
       </c>
       <c r="AH5" s="24">
         <v>125</v>
@@ -1257,14 +1243,8 @@
       <c r="AJ5" s="24">
         <v>125</v>
       </c>
-      <c r="AK5" s="24">
-        <v>62</v>
-      </c>
-      <c r="AL5" s="24">
-        <v>125</v>
-      </c>
     </row>
-    <row r="6" spans="3:38" ht="18" thickBot="1">
+    <row r="6" spans="3:36" ht="18" thickBot="1">
       <c r="C6" s="25" t="s">
         <v>43</v>
       </c>
@@ -1299,19 +1279,19 @@
         <v>182</v>
       </c>
       <c r="N6" s="21">
-        <v>146</v>
-      </c>
-      <c r="O6" s="21">
-        <v>218</v>
-      </c>
-      <c r="P6" s="21">
         <v>130</v>
       </c>
+      <c r="O6" s="22">
+        <v>386</v>
+      </c>
+      <c r="P6" s="22">
+        <v>112</v>
+      </c>
       <c r="Q6" s="22">
-        <v>386</v>
+        <v>0</v>
       </c>
       <c r="R6" s="22">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="S6" s="22">
         <v>0</v>
@@ -1320,61 +1300,55 @@
         <v>0</v>
       </c>
       <c r="U6" s="22">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="V6" s="22">
         <v>0</v>
       </c>
       <c r="W6" s="22">
-        <v>18</v>
-      </c>
-      <c r="X6" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="22">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="X6" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y6" s="23">
+        <v>78</v>
       </c>
       <c r="Z6" s="23">
         <v>156</v>
       </c>
       <c r="AA6" s="23">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="AB6" s="23">
         <v>156</v>
       </c>
       <c r="AC6" s="23">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="AD6" s="23">
-        <v>156</v>
+        <v>87</v>
       </c>
       <c r="AE6" s="23">
-        <v>109</v>
-      </c>
-      <c r="AF6" s="23">
-        <v>87</v>
-      </c>
-      <c r="AG6" s="23">
         <v>131</v>
+      </c>
+      <c r="AF6" s="24">
+        <v>125</v>
+      </c>
+      <c r="AG6" s="24">
+        <v>62</v>
       </c>
       <c r="AH6" s="24">
         <v>125</v>
       </c>
       <c r="AI6" s="24">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="AJ6" s="24">
         <v>125</v>
       </c>
-      <c r="AK6" s="24">
-        <v>75</v>
-      </c>
-      <c r="AL6" s="24">
-        <v>125</v>
-      </c>
     </row>
-    <row r="7" spans="3:38" ht="18" thickBot="1">
+    <row r="7" spans="3:36" ht="18" thickBot="1">
       <c r="C7" s="25" t="s">
         <v>44</v>
       </c>
@@ -1409,19 +1383,19 @@
         <v>208</v>
       </c>
       <c r="N7" s="21">
-        <v>166</v>
-      </c>
-      <c r="O7" s="21">
-        <v>250</v>
-      </c>
-      <c r="P7" s="21">
         <v>208</v>
       </c>
+      <c r="O7" s="22">
+        <v>657</v>
+      </c>
+      <c r="P7" s="22">
+        <v>381</v>
+      </c>
       <c r="Q7" s="22">
-        <v>657</v>
+        <v>0</v>
       </c>
       <c r="R7" s="22">
-        <v>381</v>
+        <v>0</v>
       </c>
       <c r="S7" s="22">
         <v>0</v>
@@ -1430,61 +1404,55 @@
         <v>0</v>
       </c>
       <c r="U7" s="22">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="V7" s="22">
         <v>0</v>
       </c>
       <c r="W7" s="22">
-        <v>55</v>
-      </c>
-      <c r="X7" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="22">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="X7" s="23">
+        <v>47</v>
+      </c>
+      <c r="Y7" s="23">
+        <v>23</v>
       </c>
       <c r="Z7" s="23">
-        <v>47</v>
+        <v>156</v>
       </c>
       <c r="AA7" s="23">
-        <v>23</v>
+        <v>109</v>
       </c>
       <c r="AB7" s="23">
         <v>156</v>
       </c>
       <c r="AC7" s="23">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="AD7" s="23">
-        <v>156</v>
+        <v>100</v>
       </c>
       <c r="AE7" s="23">
+        <v>150</v>
+      </c>
+      <c r="AF7" s="24">
+        <v>37</v>
+      </c>
+      <c r="AG7" s="24">
+        <v>19</v>
+      </c>
+      <c r="AH7" s="24">
         <v>125</v>
       </c>
-      <c r="AF7" s="23">
-        <v>100</v>
-      </c>
-      <c r="AG7" s="23">
-        <v>150</v>
-      </c>
-      <c r="AH7" s="24">
-        <v>37</v>
-      </c>
       <c r="AI7" s="24">
-        <v>19</v>
+        <v>87</v>
       </c>
       <c r="AJ7" s="24">
         <v>125</v>
       </c>
-      <c r="AK7" s="24">
-        <v>87</v>
-      </c>
-      <c r="AL7" s="24">
-        <v>125</v>
-      </c>
     </row>
-    <row r="8" spans="3:38" ht="18" thickBot="1">
+    <row r="8" spans="3:36" ht="18" thickBot="1">
       <c r="C8" s="25" t="s">
         <v>45</v>
       </c>
@@ -1519,82 +1487,76 @@
         <v>130</v>
       </c>
       <c r="N8" s="21">
-        <v>130</v>
-      </c>
-      <c r="O8" s="21">
         <v>195</v>
       </c>
-      <c r="P8" s="21">
-        <v>195</v>
+      <c r="O8" s="22">
+        <v>1386</v>
+      </c>
+      <c r="P8" s="22">
+        <v>1040</v>
       </c>
       <c r="Q8" s="22">
-        <v>1386</v>
+        <v>59</v>
       </c>
       <c r="R8" s="22">
-        <v>1040</v>
+        <v>1078</v>
       </c>
       <c r="S8" s="22">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="T8" s="22">
-        <v>1078</v>
+        <v>664</v>
       </c>
       <c r="U8" s="22">
-        <v>0</v>
+        <v>325</v>
       </c>
       <c r="V8" s="22">
-        <v>664</v>
+        <v>227</v>
       </c>
       <c r="W8" s="22">
-        <v>325</v>
-      </c>
-      <c r="X8" s="22">
-        <v>227</v>
-      </c>
-      <c r="Y8" s="22">
         <v>189</v>
       </c>
+      <c r="X8" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y8" s="23">
+        <v>234</v>
+      </c>
       <c r="Z8" s="23">
-        <v>156</v>
+        <v>117</v>
       </c>
       <c r="AA8" s="23">
-        <v>234</v>
+        <v>78</v>
       </c>
       <c r="AB8" s="23">
+        <v>78</v>
+      </c>
+      <c r="AC8" s="23">
+        <v>78</v>
+      </c>
+      <c r="AD8" s="23">
+        <v>78</v>
+      </c>
+      <c r="AE8" s="23">
         <v>117</v>
       </c>
-      <c r="AC8" s="23">
-        <v>78</v>
-      </c>
-      <c r="AD8" s="23">
-        <v>78</v>
-      </c>
-      <c r="AE8" s="23">
-        <v>78</v>
-      </c>
-      <c r="AF8" s="23">
-        <v>78</v>
-      </c>
-      <c r="AG8" s="23">
-        <v>117</v>
+      <c r="AF8" s="24">
+        <v>125</v>
+      </c>
+      <c r="AG8" s="24">
+        <v>187</v>
       </c>
       <c r="AH8" s="24">
-        <v>125</v>
+        <v>94</v>
       </c>
       <c r="AI8" s="24">
-        <v>187</v>
+        <v>62</v>
       </c>
       <c r="AJ8" s="24">
-        <v>94</v>
-      </c>
-      <c r="AK8" s="24">
-        <v>62</v>
-      </c>
-      <c r="AL8" s="24">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="3:38" ht="18" thickBot="1">
+    <row r="9" spans="3:36" ht="18" thickBot="1">
       <c r="C9" s="25" t="s">
         <v>46</v>
       </c>
@@ -1629,82 +1591,76 @@
         <v>390</v>
       </c>
       <c r="N9" s="21">
-        <v>312</v>
-      </c>
-      <c r="O9" s="21">
-        <v>130</v>
-      </c>
-      <c r="P9" s="21">
-        <v>78</v>
+        <v>78</v>
+      </c>
+      <c r="O9" s="22">
+        <v>486</v>
+      </c>
+      <c r="P9" s="22">
+        <v>352</v>
       </c>
       <c r="Q9" s="22">
-        <v>486</v>
+        <v>0</v>
       </c>
       <c r="R9" s="22">
-        <v>352</v>
+        <v>0</v>
       </c>
       <c r="S9" s="22">
         <v>0</v>
       </c>
       <c r="T9" s="22">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="U9" s="22">
         <v>0</v>
       </c>
       <c r="V9" s="22">
-        <v>97</v>
+        <v>9</v>
       </c>
       <c r="W9" s="22">
-        <v>0</v>
-      </c>
-      <c r="X9" s="22">
-        <v>9</v>
-      </c>
-      <c r="Y9" s="22">
         <v>106</v>
+      </c>
+      <c r="X9" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y9" s="23">
+        <v>16</v>
       </c>
       <c r="Z9" s="23">
         <v>156</v>
       </c>
       <c r="AA9" s="23">
-        <v>16</v>
+        <v>156</v>
       </c>
       <c r="AB9" s="23">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="AC9" s="23">
-        <v>156</v>
+        <v>234</v>
       </c>
       <c r="AD9" s="23">
-        <v>78</v>
+        <v>187</v>
       </c>
       <c r="AE9" s="23">
-        <v>234</v>
-      </c>
-      <c r="AF9" s="23">
-        <v>187</v>
-      </c>
-      <c r="AG9" s="23">
-        <v>78</v>
+        <v>78</v>
+      </c>
+      <c r="AF9" s="24">
+        <v>125</v>
+      </c>
+      <c r="AG9" s="24">
+        <v>12</v>
       </c>
       <c r="AH9" s="24">
         <v>125</v>
       </c>
       <c r="AI9" s="24">
-        <v>12</v>
+        <v>125</v>
       </c>
       <c r="AJ9" s="24">
-        <v>125</v>
-      </c>
-      <c r="AK9" s="24">
-        <v>125</v>
-      </c>
-      <c r="AL9" s="24">
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="3:38" ht="18" thickBot="1">
+    <row r="10" spans="3:36" ht="18" thickBot="1">
       <c r="C10" s="25" t="s">
         <v>47</v>
       </c>
@@ -1739,82 +1695,76 @@
         <v>226</v>
       </c>
       <c r="N10" s="21">
-        <v>182</v>
-      </c>
-      <c r="O10" s="21">
-        <v>130</v>
-      </c>
-      <c r="P10" s="21">
         <v>226</v>
       </c>
+      <c r="O10" s="22">
+        <v>1109</v>
+      </c>
+      <c r="P10" s="22">
+        <v>991</v>
+      </c>
       <c r="Q10" s="22">
-        <v>1109</v>
+        <v>0</v>
       </c>
       <c r="R10" s="22">
-        <v>991</v>
+        <v>0</v>
       </c>
       <c r="S10" s="22">
         <v>0</v>
       </c>
       <c r="T10" s="22">
-        <v>0</v>
+        <v>353</v>
       </c>
       <c r="U10" s="22">
         <v>0</v>
       </c>
       <c r="V10" s="22">
-        <v>353</v>
+        <v>0</v>
       </c>
       <c r="W10" s="22">
-        <v>0</v>
-      </c>
-      <c r="X10" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="22">
         <v>192</v>
       </c>
+      <c r="X10" s="23">
+        <v>234</v>
+      </c>
+      <c r="Y10" s="23">
+        <v>78</v>
+      </c>
       <c r="Z10" s="23">
-        <v>234</v>
+        <v>136</v>
       </c>
       <c r="AA10" s="23">
-        <v>78</v>
+        <v>156</v>
       </c>
       <c r="AB10" s="23">
+        <v>78</v>
+      </c>
+      <c r="AC10" s="23">
         <v>136</v>
       </c>
-      <c r="AC10" s="23">
-        <v>156</v>
-      </c>
       <c r="AD10" s="23">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="AE10" s="23">
-        <v>136</v>
-      </c>
-      <c r="AF10" s="23">
+        <v>78</v>
+      </c>
+      <c r="AF10" s="24">
+        <v>187</v>
+      </c>
+      <c r="AG10" s="24">
+        <v>62</v>
+      </c>
+      <c r="AH10" s="24">
         <v>109</v>
       </c>
-      <c r="AG10" s="23">
-        <v>78</v>
-      </c>
-      <c r="AH10" s="24">
-        <v>187</v>
-      </c>
       <c r="AI10" s="24">
-        <v>62</v>
+        <v>125</v>
       </c>
       <c r="AJ10" s="24">
-        <v>109</v>
-      </c>
-      <c r="AK10" s="24">
-        <v>125</v>
-      </c>
-      <c r="AL10" s="24">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="3:38" ht="18" thickBot="1">
+    <row r="11" spans="3:36" ht="18" thickBot="1">
       <c r="C11" s="25" t="s">
         <v>48</v>
       </c>
@@ -1849,82 +1799,76 @@
         <v>130</v>
       </c>
       <c r="N11" s="21">
-        <v>260</v>
-      </c>
-      <c r="O11" s="21">
-        <v>390</v>
-      </c>
-      <c r="P11" s="21">
-        <v>78</v>
+        <v>78</v>
+      </c>
+      <c r="O11" s="22">
+        <v>2808</v>
+      </c>
+      <c r="P11" s="22">
+        <v>1950</v>
       </c>
       <c r="Q11" s="22">
-        <v>2808</v>
+        <v>142</v>
       </c>
       <c r="R11" s="22">
-        <v>1950</v>
+        <v>1525</v>
       </c>
       <c r="S11" s="22">
-        <v>142</v>
+        <v>0</v>
       </c>
       <c r="T11" s="22">
-        <v>1525</v>
+        <v>591</v>
       </c>
       <c r="U11" s="22">
-        <v>0</v>
+        <v>532</v>
       </c>
       <c r="V11" s="22">
-        <v>591</v>
+        <v>322</v>
       </c>
       <c r="W11" s="22">
         <v>532</v>
       </c>
-      <c r="X11" s="22">
-        <v>322</v>
-      </c>
-      <c r="Y11" s="22">
-        <v>532</v>
+      <c r="X11" s="23">
+        <v>468</v>
+      </c>
+      <c r="Y11" s="23">
+        <v>78</v>
       </c>
       <c r="Z11" s="23">
-        <v>468</v>
+        <v>156</v>
       </c>
       <c r="AA11" s="23">
-        <v>78</v>
+        <v>156</v>
       </c>
       <c r="AB11" s="23">
+        <v>78</v>
+      </c>
+      <c r="AC11" s="23">
+        <v>78</v>
+      </c>
+      <c r="AD11" s="23">
         <v>156</v>
       </c>
-      <c r="AC11" s="23">
-        <v>156</v>
-      </c>
-      <c r="AD11" s="23">
-        <v>78</v>
-      </c>
       <c r="AE11" s="23">
-        <v>78</v>
-      </c>
-      <c r="AF11" s="23">
-        <v>156</v>
-      </c>
-      <c r="AG11" s="23">
         <v>234</v>
       </c>
+      <c r="AF11" s="24">
+        <v>374</v>
+      </c>
+      <c r="AG11" s="24">
+        <v>62</v>
+      </c>
       <c r="AH11" s="24">
-        <v>374</v>
+        <v>125</v>
       </c>
       <c r="AI11" s="24">
-        <v>62</v>
+        <v>125</v>
       </c>
       <c r="AJ11" s="24">
-        <v>125</v>
-      </c>
-      <c r="AK11" s="24">
-        <v>125</v>
-      </c>
-      <c r="AL11" s="24">
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="3:38" ht="18" thickBot="1">
+    <row r="12" spans="3:36" ht="18" thickBot="1">
       <c r="C12" s="25" t="s">
         <v>49</v>
       </c>
@@ -1959,82 +1903,76 @@
         <v>65</v>
       </c>
       <c r="N12" s="21">
-        <v>130</v>
-      </c>
-      <c r="O12" s="21">
-        <v>195</v>
-      </c>
-      <c r="P12" s="21">
         <v>65</v>
       </c>
+      <c r="O12" s="22">
+        <v>1908</v>
+      </c>
+      <c r="P12" s="22">
+        <v>1571</v>
+      </c>
       <c r="Q12" s="22">
-        <v>1908</v>
+        <v>93</v>
       </c>
       <c r="R12" s="22">
-        <v>1571</v>
+        <v>1394</v>
       </c>
       <c r="S12" s="22">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="T12" s="22">
-        <v>1394</v>
+        <v>431</v>
       </c>
       <c r="U12" s="22">
-        <v>0</v>
+        <v>435</v>
       </c>
       <c r="V12" s="22">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="W12" s="22">
-        <v>435</v>
-      </c>
-      <c r="X12" s="22">
-        <v>425</v>
-      </c>
-      <c r="Y12" s="22">
         <v>6</v>
       </c>
+      <c r="X12" s="23">
+        <v>468</v>
+      </c>
+      <c r="Y12" s="23">
+        <v>78</v>
+      </c>
       <c r="Z12" s="23">
-        <v>468</v>
+        <v>39</v>
       </c>
       <c r="AA12" s="23">
-        <v>78</v>
+        <v>234</v>
       </c>
       <c r="AB12" s="23">
+        <v>47</v>
+      </c>
+      <c r="AC12" s="23">
         <v>39</v>
       </c>
-      <c r="AC12" s="23">
-        <v>234</v>
-      </c>
       <c r="AD12" s="23">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="AE12" s="23">
-        <v>39</v>
-      </c>
-      <c r="AF12" s="23">
-        <v>78</v>
-      </c>
-      <c r="AG12" s="23">
         <v>117</v>
       </c>
+      <c r="AF12" s="24">
+        <v>374</v>
+      </c>
+      <c r="AG12" s="24">
+        <v>62</v>
+      </c>
       <c r="AH12" s="24">
-        <v>374</v>
+        <v>31</v>
       </c>
       <c r="AI12" s="24">
-        <v>62</v>
+        <v>187</v>
       </c>
       <c r="AJ12" s="24">
-        <v>31</v>
-      </c>
-      <c r="AK12" s="24">
-        <v>187</v>
-      </c>
-      <c r="AL12" s="24">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="3:38" ht="18" thickBot="1">
+    <row r="13" spans="3:36" ht="18" thickBot="1">
       <c r="C13" s="25" t="s">
         <v>50</v>
       </c>
@@ -2069,82 +2007,76 @@
         <v>65</v>
       </c>
       <c r="N13" s="21">
-        <v>260</v>
-      </c>
-      <c r="O13" s="21">
-        <v>390</v>
-      </c>
-      <c r="P13" s="21">
         <v>65</v>
       </c>
+      <c r="O13" s="22">
+        <v>1029</v>
+      </c>
+      <c r="P13" s="22">
+        <v>816</v>
+      </c>
       <c r="Q13" s="22">
-        <v>1029</v>
+        <v>0</v>
       </c>
       <c r="R13" s="22">
-        <v>816</v>
+        <v>224</v>
       </c>
       <c r="S13" s="22">
         <v>0</v>
       </c>
       <c r="T13" s="22">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="U13" s="22">
         <v>0</v>
       </c>
       <c r="V13" s="22">
-        <v>215</v>
+        <v>0</v>
       </c>
       <c r="W13" s="22">
-        <v>0</v>
-      </c>
-      <c r="X13" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y13" s="22">
         <v>2</v>
       </c>
+      <c r="X13" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y13" s="23">
+        <v>78</v>
+      </c>
       <c r="Z13" s="23">
+        <v>39</v>
+      </c>
+      <c r="AA13" s="23">
+        <v>78</v>
+      </c>
+      <c r="AB13" s="23">
+        <v>47</v>
+      </c>
+      <c r="AC13" s="23">
+        <v>39</v>
+      </c>
+      <c r="AD13" s="23">
         <v>156</v>
       </c>
-      <c r="AA13" s="23">
-        <v>78</v>
-      </c>
-      <c r="AB13" s="23">
-        <v>39</v>
-      </c>
-      <c r="AC13" s="23">
-        <v>78</v>
-      </c>
-      <c r="AD13" s="23">
-        <v>47</v>
-      </c>
       <c r="AE13" s="23">
-        <v>39</v>
-      </c>
-      <c r="AF13" s="23">
-        <v>156</v>
-      </c>
-      <c r="AG13" s="23">
         <v>234</v>
       </c>
+      <c r="AF13" s="24">
+        <v>125</v>
+      </c>
+      <c r="AG13" s="24">
+        <v>62</v>
+      </c>
       <c r="AH13" s="24">
-        <v>125</v>
+        <v>31</v>
       </c>
       <c r="AI13" s="24">
         <v>62</v>
       </c>
       <c r="AJ13" s="24">
-        <v>31</v>
-      </c>
-      <c r="AK13" s="24">
-        <v>62</v>
-      </c>
-      <c r="AL13" s="24">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="3:38" ht="18" thickBot="1">
+    <row r="14" spans="3:36" ht="18" thickBot="1">
       <c r="C14" s="25" t="s">
         <v>51</v>
       </c>
@@ -2179,82 +2111,76 @@
         <v>65</v>
       </c>
       <c r="N14" s="21">
-        <v>130</v>
-      </c>
-      <c r="O14" s="21">
-        <v>195</v>
-      </c>
-      <c r="P14" s="21">
         <v>65</v>
       </c>
+      <c r="O14" s="22">
+        <v>3400</v>
+      </c>
+      <c r="P14" s="22">
+        <v>2054</v>
+      </c>
       <c r="Q14" s="22">
-        <v>3400</v>
+        <v>104</v>
       </c>
       <c r="R14" s="22">
-        <v>2054</v>
+        <v>2005</v>
       </c>
       <c r="S14" s="22">
-        <v>104</v>
+        <v>0</v>
       </c>
       <c r="T14" s="22">
-        <v>2005</v>
+        <v>599</v>
       </c>
       <c r="U14" s="22">
-        <v>0</v>
+        <v>443</v>
       </c>
       <c r="V14" s="22">
-        <v>599</v>
+        <v>179</v>
       </c>
       <c r="W14" s="22">
-        <v>443</v>
-      </c>
-      <c r="X14" s="22">
-        <v>179</v>
-      </c>
-      <c r="Y14" s="22">
         <v>291</v>
       </c>
+      <c r="X14" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y14" s="23">
+        <v>78</v>
+      </c>
       <c r="Z14" s="23">
-        <v>156</v>
+        <v>39</v>
       </c>
       <c r="AA14" s="23">
         <v>78</v>
       </c>
       <c r="AB14" s="23">
+        <v>47</v>
+      </c>
+      <c r="AC14" s="23">
         <v>39</v>
       </c>
-      <c r="AC14" s="23">
-        <v>78</v>
-      </c>
       <c r="AD14" s="23">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="AE14" s="23">
-        <v>39</v>
-      </c>
-      <c r="AF14" s="23">
-        <v>78</v>
-      </c>
-      <c r="AG14" s="23">
         <v>117</v>
       </c>
+      <c r="AF14" s="24">
+        <v>125</v>
+      </c>
+      <c r="AG14" s="24">
+        <v>62</v>
+      </c>
       <c r="AH14" s="24">
-        <v>125</v>
+        <v>31</v>
       </c>
       <c r="AI14" s="24">
         <v>62</v>
       </c>
       <c r="AJ14" s="24">
-        <v>31</v>
-      </c>
-      <c r="AK14" s="24">
-        <v>62</v>
-      </c>
-      <c r="AL14" s="24">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="3:38" ht="18" thickBot="1">
+    <row r="15" spans="3:36" ht="18" thickBot="1">
       <c r="C15" s="25" t="s">
         <v>52</v>
       </c>
@@ -2289,80 +2215,74 @@
         <v>65</v>
       </c>
       <c r="N15" s="21">
-        <v>52</v>
-      </c>
-      <c r="O15" s="21">
-        <v>78</v>
-      </c>
-      <c r="P15" s="21">
         <v>65</v>
       </c>
+      <c r="O15" s="22">
+        <v>200</v>
+      </c>
+      <c r="P15" s="22">
+        <v>150</v>
+      </c>
       <c r="Q15" s="22">
+        <v>50</v>
+      </c>
+      <c r="R15" s="22">
+        <v>1000</v>
+      </c>
+      <c r="S15" s="26"/>
+      <c r="T15" s="22">
+        <v>300</v>
+      </c>
+      <c r="U15" s="22">
         <v>200</v>
       </c>
-      <c r="R15" s="22">
+      <c r="V15" s="22">
+        <v>100</v>
+      </c>
+      <c r="W15" s="22">
         <v>150</v>
       </c>
-      <c r="S15" s="22">
-        <v>50</v>
-      </c>
-      <c r="T15" s="22">
-        <v>1000</v>
-      </c>
-      <c r="U15" s="26"/>
-      <c r="V15" s="22">
-        <v>300</v>
-      </c>
-      <c r="W15" s="22">
-        <v>200</v>
-      </c>
-      <c r="X15" s="22">
-        <v>100</v>
-      </c>
-      <c r="Y15" s="22">
-        <v>150</v>
+      <c r="X15" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y15" s="23">
+        <v>78</v>
       </c>
       <c r="Z15" s="23">
-        <v>156</v>
+        <v>39</v>
       </c>
       <c r="AA15" s="23">
         <v>78</v>
       </c>
       <c r="AB15" s="23">
+        <v>47</v>
+      </c>
+      <c r="AC15" s="23">
         <v>39</v>
       </c>
-      <c r="AC15" s="23">
-        <v>78</v>
-      </c>
       <c r="AD15" s="23">
+        <v>31</v>
+      </c>
+      <c r="AE15" s="23">
         <v>47</v>
       </c>
-      <c r="AE15" s="23">
-        <v>39</v>
-      </c>
-      <c r="AF15" s="23">
+      <c r="AF15" s="24">
+        <v>125</v>
+      </c>
+      <c r="AG15" s="24">
+        <v>62</v>
+      </c>
+      <c r="AH15" s="24">
         <v>31</v>
       </c>
-      <c r="AG15" s="23">
-        <v>47</v>
-      </c>
-      <c r="AH15" s="24">
-        <v>125</v>
-      </c>
       <c r="AI15" s="24">
         <v>62</v>
       </c>
       <c r="AJ15" s="24">
-        <v>31</v>
-      </c>
-      <c r="AK15" s="24">
-        <v>62</v>
-      </c>
-      <c r="AL15" s="24">
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="3:38" ht="18" thickBot="1">
+    <row r="16" spans="3:36" ht="18" thickBot="1">
       <c r="C16" s="25" t="s">
         <v>53</v>
       </c>
@@ -2397,82 +2317,76 @@
         <v>260</v>
       </c>
       <c r="N16" s="21">
-        <v>208</v>
-      </c>
-      <c r="O16" s="21">
-        <v>312</v>
-      </c>
-      <c r="P16" s="21">
         <v>52</v>
       </c>
+      <c r="O16" s="22">
+        <v>81</v>
+      </c>
+      <c r="P16" s="22">
+        <v>100</v>
+      </c>
       <c r="Q16" s="22">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="R16" s="22">
-        <v>100</v>
+        <v>198</v>
       </c>
       <c r="S16" s="22">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="T16" s="22">
-        <v>198</v>
+        <v>0</v>
       </c>
       <c r="U16" s="22">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="V16" s="22">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="W16" s="22">
-        <v>92</v>
-      </c>
-      <c r="X16" s="22">
-        <v>92</v>
-      </c>
-      <c r="Y16" s="22">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="X16" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y16" s="23">
+        <v>62</v>
       </c>
       <c r="Z16" s="23">
+        <v>31</v>
+      </c>
+      <c r="AA16" s="23">
+        <v>78</v>
+      </c>
+      <c r="AB16" s="23">
+        <v>47</v>
+      </c>
+      <c r="AC16" s="23">
         <v>156</v>
       </c>
-      <c r="AA16" s="23">
-        <v>62</v>
-      </c>
-      <c r="AB16" s="23">
-        <v>31</v>
-      </c>
-      <c r="AC16" s="23">
-        <v>78</v>
-      </c>
       <c r="AD16" s="23">
-        <v>47</v>
+        <v>125</v>
       </c>
       <c r="AE16" s="23">
-        <v>156</v>
-      </c>
-      <c r="AF16" s="23">
+        <v>187</v>
+      </c>
+      <c r="AF16" s="24">
         <v>125</v>
       </c>
-      <c r="AG16" s="23">
-        <v>187</v>
+      <c r="AG16" s="24">
+        <v>50</v>
       </c>
       <c r="AH16" s="24">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="AI16" s="24">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="AJ16" s="24">
-        <v>25</v>
-      </c>
-      <c r="AK16" s="24">
-        <v>62</v>
-      </c>
-      <c r="AL16" s="24">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="3:38" ht="18" thickBot="1">
+    <row r="17" spans="3:36" ht="18" thickBot="1">
       <c r="C17" s="25" t="s">
         <v>54</v>
       </c>
@@ -2507,82 +2421,76 @@
         <v>260</v>
       </c>
       <c r="N17" s="21">
-        <v>208</v>
-      </c>
-      <c r="O17" s="21">
-        <v>312</v>
-      </c>
-      <c r="P17" s="21">
         <v>52</v>
       </c>
+      <c r="O17" s="22">
+        <v>200</v>
+      </c>
+      <c r="P17" s="22">
+        <v>100</v>
+      </c>
       <c r="Q17" s="22">
+        <v>30</v>
+      </c>
+      <c r="R17" s="22">
+        <v>400</v>
+      </c>
+      <c r="S17" s="22">
+        <v>0</v>
+      </c>
+      <c r="T17" s="22">
+        <v>0</v>
+      </c>
+      <c r="U17" s="22">
         <v>200</v>
       </c>
-      <c r="R17" s="22">
-        <v>100</v>
-      </c>
-      <c r="S17" s="22">
-        <v>30</v>
-      </c>
-      <c r="T17" s="22">
-        <v>400</v>
-      </c>
-      <c r="U17" s="22">
-        <v>0</v>
-      </c>
       <c r="V17" s="22">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="W17" s="22">
-        <v>200</v>
-      </c>
-      <c r="X17" s="22">
-        <v>200</v>
-      </c>
-      <c r="Y17" s="22">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="X17" s="23">
+        <v>156</v>
+      </c>
+      <c r="Y17" s="23">
+        <v>62</v>
       </c>
       <c r="Z17" s="23">
+        <v>31</v>
+      </c>
+      <c r="AA17" s="23">
+        <v>78</v>
+      </c>
+      <c r="AB17" s="23">
+        <v>47</v>
+      </c>
+      <c r="AC17" s="23">
         <v>156</v>
       </c>
-      <c r="AA17" s="23">
-        <v>62</v>
-      </c>
-      <c r="AB17" s="23">
-        <v>31</v>
-      </c>
-      <c r="AC17" s="23">
-        <v>78</v>
-      </c>
       <c r="AD17" s="23">
-        <v>47</v>
+        <v>125</v>
       </c>
       <c r="AE17" s="23">
-        <v>156</v>
-      </c>
-      <c r="AF17" s="23">
+        <v>187</v>
+      </c>
+      <c r="AF17" s="24">
         <v>125</v>
       </c>
-      <c r="AG17" s="23">
-        <v>187</v>
+      <c r="AG17" s="24">
+        <v>50</v>
       </c>
       <c r="AH17" s="24">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="AI17" s="24">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="AJ17" s="24">
-        <v>25</v>
-      </c>
-      <c r="AK17" s="24">
-        <v>62</v>
-      </c>
-      <c r="AL17" s="24">
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="3:38" ht="18" thickBot="1">
+    <row r="18" spans="3:36" ht="18" thickBot="1">
       <c r="C18" s="25" t="s">
         <v>55</v>
       </c>
@@ -2617,82 +2525,76 @@
         <v>52</v>
       </c>
       <c r="N18" s="21">
-        <v>42</v>
-      </c>
-      <c r="O18" s="21">
-        <v>62</v>
-      </c>
-      <c r="P18" s="21">
         <v>52</v>
       </c>
+      <c r="O18" s="22">
+        <v>1017</v>
+      </c>
+      <c r="P18" s="22">
+        <v>851</v>
+      </c>
       <c r="Q18" s="22">
-        <v>1017</v>
+        <v>0</v>
       </c>
       <c r="R18" s="22">
-        <v>851</v>
+        <v>293</v>
       </c>
       <c r="S18" s="22">
         <v>0</v>
       </c>
       <c r="T18" s="22">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="U18" s="22">
         <v>0</v>
       </c>
       <c r="V18" s="22">
-        <v>287</v>
+        <v>0</v>
       </c>
       <c r="W18" s="22">
         <v>0</v>
       </c>
-      <c r="X18" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="22">
-        <v>0</v>
+      <c r="X18" s="23">
+        <v>78</v>
+      </c>
+      <c r="Y18" s="23">
+        <v>62</v>
       </c>
       <c r="Z18" s="23">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="AA18" s="23">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="AB18" s="23">
+        <v>47</v>
+      </c>
+      <c r="AC18" s="23">
         <v>31</v>
       </c>
-      <c r="AC18" s="23">
-        <v>34</v>
-      </c>
       <c r="AD18" s="23">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="AE18" s="23">
-        <v>31</v>
-      </c>
-      <c r="AF18" s="23">
+        <v>37</v>
+      </c>
+      <c r="AF18" s="24">
+        <v>62</v>
+      </c>
+      <c r="AG18" s="24">
+        <v>50</v>
+      </c>
+      <c r="AH18" s="24">
         <v>25</v>
       </c>
-      <c r="AG18" s="23">
+      <c r="AI18" s="24">
+        <v>27</v>
+      </c>
+      <c r="AJ18" s="24">
         <v>37</v>
       </c>
-      <c r="AH18" s="24">
-        <v>62</v>
-      </c>
-      <c r="AI18" s="24">
-        <v>50</v>
-      </c>
-      <c r="AJ18" s="24">
-        <v>25</v>
-      </c>
-      <c r="AK18" s="24">
-        <v>27</v>
-      </c>
-      <c r="AL18" s="24">
-        <v>37</v>
-      </c>
     </row>
-    <row r="19" spans="3:38" ht="18" thickBot="1">
+    <row r="19" spans="3:36" ht="18" thickBot="1">
       <c r="C19" s="25" t="s">
         <v>56</v>
       </c>
@@ -2727,19 +2629,19 @@
         <v>52</v>
       </c>
       <c r="N19" s="21">
-        <v>42</v>
-      </c>
-      <c r="O19" s="21">
-        <v>62</v>
-      </c>
-      <c r="P19" s="21">
         <v>52</v>
       </c>
+      <c r="O19" s="22">
+        <v>500</v>
+      </c>
+      <c r="P19" s="22">
+        <v>400</v>
+      </c>
       <c r="Q19" s="22">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="R19" s="22">
-        <v>400</v>
+        <v>150</v>
       </c>
       <c r="S19" s="22">
         <v>0</v>
@@ -2751,58 +2653,52 @@
         <v>0</v>
       </c>
       <c r="V19" s="22">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="W19" s="22">
         <v>0</v>
       </c>
-      <c r="X19" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y19" s="22">
-        <v>0</v>
+      <c r="X19" s="23">
+        <v>78</v>
+      </c>
+      <c r="Y19" s="23">
+        <v>62</v>
       </c>
       <c r="Z19" s="23">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="AA19" s="23">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="AB19" s="23">
+        <v>47</v>
+      </c>
+      <c r="AC19" s="23">
         <v>31</v>
       </c>
-      <c r="AC19" s="23">
-        <v>34</v>
-      </c>
       <c r="AD19" s="23">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="AE19" s="23">
-        <v>31</v>
-      </c>
-      <c r="AF19" s="23">
+        <v>37</v>
+      </c>
+      <c r="AF19" s="24">
+        <v>62</v>
+      </c>
+      <c r="AG19" s="24">
+        <v>50</v>
+      </c>
+      <c r="AH19" s="24">
         <v>25</v>
       </c>
-      <c r="AG19" s="23">
+      <c r="AI19" s="24">
+        <v>27</v>
+      </c>
+      <c r="AJ19" s="24">
         <v>37</v>
       </c>
-      <c r="AH19" s="24">
-        <v>62</v>
-      </c>
-      <c r="AI19" s="24">
-        <v>50</v>
-      </c>
-      <c r="AJ19" s="24">
-        <v>25</v>
-      </c>
-      <c r="AK19" s="24">
-        <v>27</v>
-      </c>
-      <c r="AL19" s="24">
-        <v>37</v>
-      </c>
     </row>
-    <row r="20" spans="3:38" ht="18" thickBot="1">
+    <row r="20" spans="3:36" ht="18" thickBot="1">
       <c r="C20" s="25" t="s">
         <v>57</v>
       </c>
@@ -2839,17 +2735,17 @@
       <c r="N20" s="21">
         <v>52</v>
       </c>
-      <c r="O20" s="21">
-        <v>78</v>
-      </c>
-      <c r="P20" s="21">
-        <v>52</v>
+      <c r="O20" s="22">
+        <v>250</v>
+      </c>
+      <c r="P20" s="22">
+        <v>200</v>
       </c>
       <c r="Q20" s="22">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="R20" s="22">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="S20" s="22">
         <v>0</v>
@@ -2861,58 +2757,52 @@
         <v>0</v>
       </c>
       <c r="V20" s="22">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="W20" s="22">
         <v>0</v>
       </c>
-      <c r="X20" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y20" s="22">
-        <v>0</v>
+      <c r="X20" s="23">
+        <v>78</v>
+      </c>
+      <c r="Y20" s="23">
+        <v>47</v>
       </c>
       <c r="Z20" s="23">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="AA20" s="23">
+        <v>31</v>
+      </c>
+      <c r="AB20" s="23">
         <v>47</v>
-      </c>
-      <c r="AB20" s="23">
-        <v>31</v>
       </c>
       <c r="AC20" s="23">
         <v>31</v>
       </c>
       <c r="AD20" s="23">
+        <v>31</v>
+      </c>
+      <c r="AE20" s="23">
         <v>47</v>
       </c>
-      <c r="AE20" s="23">
-        <v>31</v>
-      </c>
-      <c r="AF20" s="23">
-        <v>31</v>
-      </c>
-      <c r="AG20" s="23">
-        <v>47</v>
+      <c r="AF20" s="24">
+        <v>62</v>
+      </c>
+      <c r="AG20" s="24">
+        <v>37</v>
       </c>
       <c r="AH20" s="24">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="AI20" s="24">
+        <v>25</v>
+      </c>
+      <c r="AJ20" s="24">
         <v>37</v>
       </c>
-      <c r="AJ20" s="24">
-        <v>25</v>
-      </c>
-      <c r="AK20" s="24">
-        <v>25</v>
-      </c>
-      <c r="AL20" s="24">
-        <v>37</v>
-      </c>
     </row>
-    <row r="21" spans="3:38" ht="18" thickBot="1">
+    <row r="21" spans="3:36" ht="18" thickBot="1">
       <c r="C21" s="25" t="s">
         <v>58</v>
       </c>
@@ -2947,19 +2837,19 @@
         <v>52</v>
       </c>
       <c r="N21" s="21">
-        <v>42</v>
-      </c>
-      <c r="O21" s="21">
-        <v>130</v>
-      </c>
-      <c r="P21" s="21">
         <v>52</v>
       </c>
+      <c r="O21" s="22">
+        <v>100</v>
+      </c>
+      <c r="P21" s="22">
+        <v>100</v>
+      </c>
       <c r="Q21" s="22">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R21" s="22">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="S21" s="22">
         <v>0</v>
@@ -2971,58 +2861,52 @@
         <v>0</v>
       </c>
       <c r="V21" s="22">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="W21" s="22">
         <v>0</v>
       </c>
-      <c r="X21" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="22">
-        <v>0</v>
+      <c r="X21" s="23">
+        <v>78</v>
+      </c>
+      <c r="Y21" s="23">
+        <v>62</v>
       </c>
       <c r="Z21" s="23">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="AA21" s="23">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="AB21" s="23">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="AC21" s="23">
         <v>31</v>
       </c>
       <c r="AD21" s="23">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="AE21" s="23">
-        <v>31</v>
-      </c>
-      <c r="AF21" s="23">
+        <v>78</v>
+      </c>
+      <c r="AF21" s="24">
+        <v>62</v>
+      </c>
+      <c r="AG21" s="24">
+        <v>50</v>
+      </c>
+      <c r="AH21" s="24">
         <v>25</v>
       </c>
-      <c r="AG21" s="23">
-        <v>78</v>
-      </c>
-      <c r="AH21" s="24">
-        <v>62</v>
-      </c>
       <c r="AI21" s="24">
+        <v>25</v>
+      </c>
+      <c r="AJ21" s="24">
         <v>50</v>
       </c>
-      <c r="AJ21" s="24">
-        <v>25</v>
-      </c>
-      <c r="AK21" s="24">
-        <v>25</v>
-      </c>
-      <c r="AL21" s="24">
-        <v>50</v>
-      </c>
     </row>
-    <row r="22" spans="3:38" ht="18" thickBot="1">
+    <row r="22" spans="3:36" ht="18" thickBot="1">
       <c r="C22" s="25" t="s">
         <v>59</v>
       </c>
@@ -3057,82 +2941,76 @@
         <v>52</v>
       </c>
       <c r="N22" s="21">
-        <v>130</v>
-      </c>
-      <c r="O22" s="21">
-        <v>195</v>
-      </c>
-      <c r="P22" s="21">
         <v>52</v>
       </c>
+      <c r="O22" s="22">
+        <v>1314</v>
+      </c>
+      <c r="P22" s="22">
+        <v>756</v>
+      </c>
       <c r="Q22" s="22">
-        <v>1314</v>
+        <v>0</v>
       </c>
       <c r="R22" s="22">
-        <v>756</v>
+        <v>0</v>
       </c>
       <c r="S22" s="22">
-        <v>0</v>
+        <v>329</v>
       </c>
       <c r="T22" s="22">
-        <v>0</v>
+        <v>372</v>
       </c>
       <c r="U22" s="22">
-        <v>329</v>
+        <v>0</v>
       </c>
       <c r="V22" s="22">
-        <v>372</v>
+        <v>0</v>
       </c>
       <c r="W22" s="22">
         <v>0</v>
       </c>
-      <c r="X22" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="22">
-        <v>0</v>
+      <c r="X22" s="23">
+        <v>78</v>
+      </c>
+      <c r="Y22" s="23">
+        <v>62</v>
       </c>
       <c r="Z22" s="23">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="AA22" s="23">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="AB22" s="23">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="AC22" s="23">
         <v>31</v>
       </c>
       <c r="AD22" s="23">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="AE22" s="23">
-        <v>31</v>
-      </c>
-      <c r="AF22" s="23">
-        <v>78</v>
-      </c>
-      <c r="AG22" s="23">
         <v>117</v>
       </c>
+      <c r="AF22" s="24">
+        <v>62</v>
+      </c>
+      <c r="AG22" s="24">
+        <v>50</v>
+      </c>
       <c r="AH22" s="24">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="AI22" s="24">
+        <v>25</v>
+      </c>
+      <c r="AJ22" s="24">
         <v>50</v>
       </c>
-      <c r="AJ22" s="24">
-        <v>25</v>
-      </c>
-      <c r="AK22" s="24">
-        <v>25</v>
-      </c>
-      <c r="AL22" s="24">
-        <v>50</v>
-      </c>
     </row>
-    <row r="23" spans="3:38" ht="18" thickBot="1">
+    <row r="23" spans="3:36" ht="18" thickBot="1">
       <c r="C23" s="25" t="s">
         <v>60</v>
       </c>
@@ -3167,82 +3045,76 @@
         <v>52</v>
       </c>
       <c r="N23" s="21">
-        <v>130</v>
-      </c>
-      <c r="O23" s="21">
-        <v>195</v>
-      </c>
-      <c r="P23" s="21">
         <v>52</v>
       </c>
+      <c r="O23" s="22">
+        <v>1043</v>
+      </c>
+      <c r="P23" s="22">
+        <v>431</v>
+      </c>
       <c r="Q23" s="22">
-        <v>1043</v>
+        <v>0</v>
       </c>
       <c r="R23" s="22">
-        <v>431</v>
+        <v>0</v>
       </c>
       <c r="S23" s="22">
-        <v>0</v>
+        <v>198</v>
       </c>
       <c r="T23" s="22">
-        <v>0</v>
+        <v>215</v>
       </c>
       <c r="U23" s="22">
-        <v>198</v>
+        <v>0</v>
       </c>
       <c r="V23" s="22">
-        <v>215</v>
+        <v>0</v>
       </c>
       <c r="W23" s="22">
         <v>0</v>
       </c>
-      <c r="X23" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y23" s="22">
-        <v>0</v>
+      <c r="X23" s="23">
+        <v>78</v>
+      </c>
+      <c r="Y23" s="23">
+        <v>62</v>
       </c>
       <c r="Z23" s="23">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="AA23" s="23">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="AB23" s="23">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="AC23" s="23">
         <v>31</v>
       </c>
       <c r="AD23" s="23">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="AE23" s="23">
-        <v>31</v>
-      </c>
-      <c r="AF23" s="23">
-        <v>78</v>
-      </c>
-      <c r="AG23" s="23">
         <v>117</v>
       </c>
+      <c r="AF23" s="24">
+        <v>62</v>
+      </c>
+      <c r="AG23" s="24">
+        <v>50</v>
+      </c>
       <c r="AH23" s="24">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="AI23" s="24">
+        <v>25</v>
+      </c>
+      <c r="AJ23" s="24">
         <v>50</v>
       </c>
-      <c r="AJ23" s="24">
-        <v>25</v>
-      </c>
-      <c r="AK23" s="24">
-        <v>25</v>
-      </c>
-      <c r="AL23" s="24">
-        <v>50</v>
-      </c>
     </row>
-    <row r="24" spans="3:38" ht="18" thickBot="1">
+    <row r="24" spans="3:36" ht="18" thickBot="1">
       <c r="C24" s="25" t="s">
         <v>61</v>
       </c>
@@ -3277,82 +3149,76 @@
         <v>52</v>
       </c>
       <c r="N24" s="21">
-        <v>130</v>
-      </c>
-      <c r="O24" s="21">
-        <v>195</v>
-      </c>
-      <c r="P24" s="21">
         <v>52</v>
       </c>
+      <c r="O24" s="22">
+        <v>3226</v>
+      </c>
+      <c r="P24" s="22">
+        <v>1602</v>
+      </c>
       <c r="Q24" s="22">
-        <v>3226</v>
+        <v>44</v>
       </c>
       <c r="R24" s="22">
-        <v>1602</v>
+        <v>1872</v>
       </c>
       <c r="S24" s="22">
-        <v>44</v>
+        <v>489</v>
       </c>
       <c r="T24" s="22">
-        <v>1872</v>
+        <v>1218</v>
       </c>
       <c r="U24" s="22">
-        <v>489</v>
+        <v>452</v>
       </c>
       <c r="V24" s="22">
-        <v>1218</v>
+        <v>415</v>
       </c>
       <c r="W24" s="22">
-        <v>452</v>
-      </c>
-      <c r="X24" s="22">
-        <v>415</v>
-      </c>
-      <c r="Y24" s="22">
         <v>13</v>
       </c>
+      <c r="X24" s="23">
+        <v>78</v>
+      </c>
+      <c r="Y24" s="23">
+        <v>62</v>
+      </c>
       <c r="Z24" s="23">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="AA24" s="23">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="AB24" s="23">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="AC24" s="23">
         <v>31</v>
       </c>
       <c r="AD24" s="23">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="AE24" s="23">
-        <v>31</v>
-      </c>
-      <c r="AF24" s="23">
-        <v>78</v>
-      </c>
-      <c r="AG24" s="23">
         <v>117</v>
       </c>
+      <c r="AF24" s="24">
+        <v>62</v>
+      </c>
+      <c r="AG24" s="24">
+        <v>50</v>
+      </c>
       <c r="AH24" s="24">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="AI24" s="24">
+        <v>25</v>
+      </c>
+      <c r="AJ24" s="24">
         <v>50</v>
       </c>
-      <c r="AJ24" s="24">
-        <v>25</v>
-      </c>
-      <c r="AK24" s="24">
-        <v>25</v>
-      </c>
-      <c r="AL24" s="24">
-        <v>50</v>
-      </c>
     </row>
-    <row r="25" spans="3:38" ht="18" thickBot="1">
+    <row r="25" spans="3:36" ht="18" thickBot="1">
       <c r="C25" s="25" t="s">
         <v>62</v>
       </c>
@@ -3387,14 +3253,10 @@
         <v>130</v>
       </c>
       <c r="N25" s="21">
-        <v>104</v>
-      </c>
-      <c r="O25" s="21">
-        <v>156</v>
-      </c>
-      <c r="P25" s="21">
         <v>130</v>
       </c>
+      <c r="O25" s="26"/>
+      <c r="P25" s="26"/>
       <c r="Q25" s="26"/>
       <c r="R25" s="26"/>
       <c r="S25" s="26"/>
@@ -3402,49 +3264,47 @@
       <c r="U25" s="26"/>
       <c r="V25" s="26"/>
       <c r="W25" s="26"/>
-      <c r="X25" s="26"/>
-      <c r="Y25" s="26"/>
+      <c r="X25" s="23">
+        <v>78</v>
+      </c>
+      <c r="Y25" s="23">
+        <v>39</v>
+      </c>
       <c r="Z25" s="23">
         <v>78</v>
       </c>
       <c r="AA25" s="23">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="AB25" s="23">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="AC25" s="23">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="AD25" s="23">
         <v>62</v>
       </c>
       <c r="AE25" s="23">
-        <v>78</v>
-      </c>
-      <c r="AF25" s="23">
-        <v>62</v>
-      </c>
-      <c r="AG25" s="23">
         <v>94</v>
       </c>
+      <c r="AF25" s="24">
+        <v>62</v>
+      </c>
+      <c r="AG25" s="24">
+        <v>31</v>
+      </c>
       <c r="AH25" s="24">
         <v>62</v>
       </c>
       <c r="AI25" s="24">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="AJ25" s="24">
-        <v>62</v>
-      </c>
-      <c r="AK25" s="24">
-        <v>37</v>
-      </c>
-      <c r="AL25" s="24">
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="3:38" ht="18" thickBot="1">
+    <row r="26" spans="3:36" ht="18" thickBot="1">
       <c r="C26" s="25" t="s">
         <v>36</v>
       </c>
@@ -3463,8 +3323,8 @@
       <c r="L26" s="28"/>
       <c r="M26" s="28"/>
       <c r="N26" s="28"/>
-      <c r="O26" s="28"/>
-      <c r="P26" s="28"/>
+      <c r="O26" s="26"/>
+      <c r="P26" s="26"/>
       <c r="Q26" s="26"/>
       <c r="R26" s="26"/>
       <c r="S26" s="26"/>
@@ -3472,23 +3332,21 @@
       <c r="U26" s="26"/>
       <c r="V26" s="26"/>
       <c r="W26" s="26"/>
-      <c r="X26" s="26"/>
-      <c r="Y26" s="26"/>
+      <c r="X26" s="29"/>
+      <c r="Y26" s="29"/>
       <c r="Z26" s="29"/>
       <c r="AA26" s="29"/>
       <c r="AB26" s="29"/>
       <c r="AC26" s="29"/>
       <c r="AD26" s="29"/>
       <c r="AE26" s="29"/>
-      <c r="AF26" s="29"/>
-      <c r="AG26" s="29"/>
+      <c r="AF26" s="30"/>
+      <c r="AG26" s="30"/>
       <c r="AH26" s="30"/>
       <c r="AI26" s="30"/>
       <c r="AJ26" s="30"/>
-      <c r="AK26" s="30"/>
-      <c r="AL26" s="30"/>
     </row>
-    <row r="27" spans="3:38" ht="18" thickBot="1">
+    <row r="27" spans="3:36" ht="18" thickBot="1">
       <c r="C27" s="25" t="s">
         <v>37</v>
       </c>
@@ -3507,8 +3365,8 @@
       <c r="L27" s="28"/>
       <c r="M27" s="28"/>
       <c r="N27" s="28"/>
-      <c r="O27" s="28"/>
-      <c r="P27" s="28"/>
+      <c r="O27" s="26"/>
+      <c r="P27" s="26"/>
       <c r="Q27" s="26"/>
       <c r="R27" s="26"/>
       <c r="S27" s="26"/>
@@ -3516,23 +3374,21 @@
       <c r="U27" s="26"/>
       <c r="V27" s="26"/>
       <c r="W27" s="26"/>
-      <c r="X27" s="26"/>
-      <c r="Y27" s="26"/>
+      <c r="X27" s="29"/>
+      <c r="Y27" s="29"/>
       <c r="Z27" s="29"/>
       <c r="AA27" s="29"/>
       <c r="AB27" s="29"/>
       <c r="AC27" s="29"/>
       <c r="AD27" s="29"/>
       <c r="AE27" s="29"/>
-      <c r="AF27" s="29"/>
-      <c r="AG27" s="29"/>
+      <c r="AF27" s="30"/>
+      <c r="AG27" s="30"/>
       <c r="AH27" s="30"/>
       <c r="AI27" s="30"/>
       <c r="AJ27" s="30"/>
-      <c r="AK27" s="30"/>
-      <c r="AL27" s="30"/>
     </row>
-    <row r="28" spans="3:38" ht="18" thickBot="1">
+    <row r="28" spans="3:36" ht="18" thickBot="1">
       <c r="C28" s="25" t="s">
         <v>38</v>
       </c>
@@ -3551,8 +3407,8 @@
       <c r="L28" s="28"/>
       <c r="M28" s="28"/>
       <c r="N28" s="28"/>
-      <c r="O28" s="28"/>
-      <c r="P28" s="28"/>
+      <c r="O28" s="26"/>
+      <c r="P28" s="26"/>
       <c r="Q28" s="26"/>
       <c r="R28" s="26"/>
       <c r="S28" s="26"/>
@@ -3560,23 +3416,21 @@
       <c r="U28" s="26"/>
       <c r="V28" s="26"/>
       <c r="W28" s="26"/>
-      <c r="X28" s="26"/>
-      <c r="Y28" s="26"/>
+      <c r="X28" s="29"/>
+      <c r="Y28" s="29"/>
       <c r="Z28" s="29"/>
       <c r="AA28" s="29"/>
       <c r="AB28" s="29"/>
       <c r="AC28" s="29"/>
       <c r="AD28" s="29"/>
       <c r="AE28" s="29"/>
-      <c r="AF28" s="29"/>
-      <c r="AG28" s="29"/>
+      <c r="AF28" s="30"/>
+      <c r="AG28" s="30"/>
       <c r="AH28" s="30"/>
       <c r="AI28" s="30"/>
       <c r="AJ28" s="30"/>
-      <c r="AK28" s="30"/>
-      <c r="AL28" s="30"/>
     </row>
-    <row r="29" spans="3:38" ht="18" thickBot="1">
+    <row r="29" spans="3:36" ht="18" thickBot="1">
       <c r="C29" s="25" t="s">
         <v>39</v>
       </c>
@@ -3595,8 +3449,8 @@
       <c r="L29" s="28"/>
       <c r="M29" s="28"/>
       <c r="N29" s="28"/>
-      <c r="O29" s="28"/>
-      <c r="P29" s="28"/>
+      <c r="O29" s="26"/>
+      <c r="P29" s="26"/>
       <c r="Q29" s="26"/>
       <c r="R29" s="26"/>
       <c r="S29" s="26"/>
@@ -3604,23 +3458,21 @@
       <c r="U29" s="26"/>
       <c r="V29" s="26"/>
       <c r="W29" s="26"/>
-      <c r="X29" s="26"/>
-      <c r="Y29" s="26"/>
+      <c r="X29" s="29"/>
+      <c r="Y29" s="29"/>
       <c r="Z29" s="29"/>
       <c r="AA29" s="29"/>
       <c r="AB29" s="29"/>
       <c r="AC29" s="29"/>
       <c r="AD29" s="29"/>
       <c r="AE29" s="29"/>
-      <c r="AF29" s="29"/>
-      <c r="AG29" s="29"/>
+      <c r="AF29" s="30"/>
+      <c r="AG29" s="30"/>
       <c r="AH29" s="30"/>
       <c r="AI29" s="30"/>
       <c r="AJ29" s="30"/>
-      <c r="AK29" s="30"/>
-      <c r="AL29" s="30"/>
     </row>
-    <row r="30" spans="3:38" ht="18" thickBot="1">
+    <row r="30" spans="3:36" ht="18" thickBot="1">
       <c r="C30" s="25" t="s">
         <v>40</v>
       </c>
@@ -3639,50 +3491,48 @@
       <c r="L30" s="28"/>
       <c r="M30" s="28"/>
       <c r="N30" s="28"/>
-      <c r="O30" s="28"/>
-      <c r="P30" s="28"/>
+      <c r="O30" s="22">
+        <v>363</v>
+      </c>
+      <c r="P30" s="22">
+        <v>235</v>
+      </c>
       <c r="Q30" s="22">
-        <v>363</v>
+        <v>0</v>
       </c>
       <c r="R30" s="22">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="S30" s="22">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="T30" s="22">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="U30" s="22">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="V30" s="22">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="W30" s="22">
         <v>0</v>
       </c>
-      <c r="X30" s="22">
-        <v>0</v>
-      </c>
-      <c r="Y30" s="22">
-        <v>0</v>
-      </c>
+      <c r="X30" s="29"/>
+      <c r="Y30" s="29"/>
       <c r="Z30" s="29"/>
       <c r="AA30" s="29"/>
       <c r="AB30" s="29"/>
       <c r="AC30" s="29"/>
       <c r="AD30" s="29"/>
       <c r="AE30" s="29"/>
-      <c r="AF30" s="29"/>
-      <c r="AG30" s="29"/>
+      <c r="AF30" s="30"/>
+      <c r="AG30" s="30"/>
       <c r="AH30" s="30"/>
       <c r="AI30" s="30"/>
       <c r="AJ30" s="30"/>
-      <c r="AK30" s="30"/>
-      <c r="AL30" s="30"/>
     </row>
-    <row r="31" spans="3:38" ht="18" thickBot="1">
+    <row r="31" spans="3:36" ht="18" thickBot="1">
       <c r="C31" s="31"/>
       <c r="D31" s="32">
         <v>56250</v>
@@ -3700,37 +3550,35 @@
       <c r="K31" s="35"/>
       <c r="L31" s="35"/>
       <c r="M31" s="35"/>
-      <c r="N31" s="35"/>
-      <c r="O31" s="35"/>
-      <c r="P31" s="31"/>
-      <c r="Q31" s="36">
+      <c r="N31" s="31"/>
+      <c r="O31" s="36">
         <v>60694</v>
       </c>
+      <c r="P31" s="35"/>
+      <c r="Q31" s="35"/>
       <c r="R31" s="35"/>
       <c r="S31" s="35"/>
       <c r="T31" s="35"/>
       <c r="U31" s="35"/>
       <c r="V31" s="35"/>
-      <c r="W31" s="35"/>
-      <c r="X31" s="35"/>
-      <c r="Y31" s="31"/>
-      <c r="Z31" s="37">
+      <c r="W31" s="31"/>
+      <c r="X31" s="37">
         <v>16222</v>
       </c>
+      <c r="Y31" s="35"/>
+      <c r="Z31" s="35"/>
       <c r="AA31" s="35"/>
       <c r="AB31" s="35"/>
       <c r="AC31" s="35"/>
       <c r="AD31" s="35"/>
-      <c r="AE31" s="35"/>
-      <c r="AF31" s="35"/>
-      <c r="AG31" s="31"/>
-      <c r="AH31" s="38">
+      <c r="AE31" s="31"/>
+      <c r="AF31" s="38">
         <v>8107</v>
       </c>
+      <c r="AG31" s="35"/>
+      <c r="AH31" s="35"/>
       <c r="AI31" s="35"/>
       <c r="AJ31" s="35"/>
-      <c r="AK31" s="35"/>
-      <c r="AL31" s="35"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>